<commit_message>
Changes from OB staff feedback
</commit_message>
<xml_diff>
--- a/static/fields/drugorangebook_reference.xlsx
+++ b/static/fields/drugorangebook_reference.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10412"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/violet.wren/WebstormProjects/open.fda.gov/static/fields/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C6A34E-AB94-0242-90A5-6DC162115518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4532AD78-D231-8D4F-BA25-271332F4199E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="21900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,33 +54,15 @@
     <t>route</t>
   </si>
   <si>
-    <t>Brand or trade name of the drug product.</t>
-  </si>
-  <si>
     <t>name</t>
   </si>
   <si>
     <t>strength</t>
   </si>
   <si>
-    <t>The names of the active, medicinal ingredients in the drug product.</t>
-  </si>
-  <si>
-    <t>The strength of the active, medicinal ingredients in the drug product.</t>
-  </si>
-  <si>
     <t>dosage_form</t>
   </si>
   <si>
-    <t>The drug’s dosage form. There is no standard, but values may include terms like `tablet` or `solution for injection`.</t>
-  </si>
-  <si>
-    <t>applicant_number</t>
-  </si>
-  <si>
-    <t>applicant_full_name</t>
-  </si>
-  <si>
     <t>application_type</t>
   </si>
   <si>
@@ -105,9 +87,6 @@
     <t>patent_number</t>
   </si>
   <si>
-    <t>expire_date</t>
-  </si>
-  <si>
     <t>drug_substance_flag</t>
   </si>
   <si>
@@ -129,39 +108,15 @@
     <t>exclusivity_code</t>
   </si>
   <si>
-    <t>exclusivity_expire_date</t>
-  </si>
-  <si>
     <t>Name of the Applicant for the drug product.</t>
   </si>
   <si>
-    <t>The full name of the firm holding legal responsibility for the new drug application.</t>
-  </si>
-  <si>
-    <t>The type of new drug application approval.</t>
-  </si>
-  <si>
     <t>The FDA assigned number to the application.</t>
   </si>
   <si>
-    <t>The FDA assigned number to identify the application products. Each strength is a separate product. May repeat for multiple part products.</t>
-  </si>
-  <si>
-    <t>The TE Code indicates the therapeutic equivalence rating of generic to innovator Rx products.</t>
-  </si>
-  <si>
-    <t>The date the product was approved as stated in the FDA approval letter to the applicant.</t>
-  </si>
-  <si>
     <t>Products approved prior to the January 1, 1982 contain the phrase: "Approved prior to Jan 1, 1982".</t>
   </si>
   <si>
-    <t>The group or category of approved drugs.</t>
-  </si>
-  <si>
-    <t>Patent numbers as submitted by the applicant holder for patents covered by the statutory provisions.  May repeat for multiple applications and multiple products. Includes pediatric exclusivity granted by the agency.</t>
-  </si>
-  <si>
     <t>The date the patent expires as submitted by the applicant holder including applicable extensions.</t>
   </si>
   <si>
@@ -171,30 +126,15 @@
     <t>Patents submitted on FDA Form 3542 and listed after August 18, 2003 may have a drug product flag indicating the sponsor submitted the patent as claiming the drug product.</t>
   </si>
   <si>
-    <t>Code to designate a use patent that covers the approved indication or use of a drug product.  May repeat for multiple applications, multiple products and multiple patents.</t>
-  </si>
-  <si>
-    <t>Sponsor has requested patent be delisted. This patent has remained listed because, under Section 505(j)(5)(D)(i) of the Act, a first applicant may retain eligibility for 180-day exclusivity based on a paragraph IV certification to this patent for a certain period. Applicants under Section 505(b)(2) are not required to certify to patents where this flag is set to Y.</t>
-  </si>
-  <si>
-    <t>The date on which the FDA receives patent information from the new drug application (NDA) holder.</t>
-  </si>
-  <si>
     <t>Code to designate exclusivity granted by the FDA to a drug product.</t>
   </si>
   <si>
     <t>The date the exclusivity expires.</t>
   </si>
   <si>
-    <t>The RLD is a drug product approved under section 505(c) of the FD&amp;C Act for which FDA has made a finding of safety and effectiveness. In the electronic Orange Book, an RLD is identified by “RLD” in the RLD column.</t>
-  </si>
-  <si>
     <t>reference_standard</t>
   </si>
   <si>
-    <t>A highly purified compound that is well characterized.</t>
-  </si>
-  <si>
     <t>active_ingredients</t>
   </si>
   <si>
@@ -217,6 +157,66 @@
   </si>
   <si>
     <t>array of objects</t>
+  </si>
+  <si>
+    <t>The FDA assigned number to identify the application products.</t>
+  </si>
+  <si>
+    <t>The date the product was approved.</t>
+  </si>
+  <si>
+    <t>The name of the active drug ingredient in the drug product.</t>
+  </si>
+  <si>
+    <t>The amount of the active ingredient in the drug product.</t>
+  </si>
+  <si>
+    <t>The physical form in which a drug is manufactured or administered.</t>
+  </si>
+  <si>
+    <t>The proprietary name of the drug product.</t>
+  </si>
+  <si>
+    <t>The full name of the applicant holder.</t>
+  </si>
+  <si>
+    <t>The type of new drug application.</t>
+  </si>
+  <si>
+    <t>The code that indicates the therapeutic equivalence of a drug product to other pharmacetically equivalent products listed in the Orange Book.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The RLD is a drug product approved under section 505(c) of the FD&amp;C Act for which FDA has made a finding of safety and effectiveness. </t>
+  </si>
+  <si>
+    <t>The designated product that abbreviated new drug application (ANDA) applicants should use for bioequivalence studies.</t>
+  </si>
+  <si>
+    <t>The product type describes the marketing status of the product.</t>
+  </si>
+  <si>
+    <t>Patent numbers as submitted by the applicant holder for patents covered by the statutory provisions.  May include pediatric exclusivity granted by the agency.</t>
+  </si>
+  <si>
+    <t>A code to designate a method of use that covers the approved indication or use of a drug product.</t>
+  </si>
+  <si>
+    <t>The flag is set to "Y" when an applicant holder has requested a patent to be delisted but the patent cannot be delisted.</t>
+  </si>
+  <si>
+    <t>The date on which the FDA receives patent information from the applicant holder. Patent submission date data is included for patents submitted after 2013.</t>
+  </si>
+  <si>
+    <t>exclusivity_expiration_date</t>
+  </si>
+  <si>
+    <t>expiration_date</t>
+  </si>
+  <si>
+    <t>application_full_name</t>
+  </si>
+  <si>
+    <t>application_name</t>
   </si>
 </sst>
 </file>
@@ -387,7 +387,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -412,6 +412,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="99">
@@ -860,7 +863,7 @@
     <col min="5" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
@@ -874,103 +877,103 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B2" s="4" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>39</v>
+      <c r="D2" s="9" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>41</v>
+      <c r="D3" s="9" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="4" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="C9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>15</v>
+      <c r="D9" s="9" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>8</v>
@@ -979,12 +982,12 @@
         <v>3</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>7</v>
@@ -993,54 +996,54 @@
         <v>3</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D12" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D13" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
         <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
-        <v>57</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>6</v>
@@ -1049,54 +1052,54 @@
         <v>3</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D16" s="5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="D16" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>54</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>4</v>
@@ -1104,150 +1107,150 @@
       <c r="C19" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>43</v>
+      <c r="D19" s="9" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B20" s="4" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24" s="3" t="s">
+      <c r="C27" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" s="9" t="s">
         <v>59</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="68" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B28" s="4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B29" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B30" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>